<commit_message>
Contenidos: agregar Guiones + modo Teleprompter
- Nuevo campo "Guion" en el modal de contenido, con botón para
  abrirlo a pantalla completa (fondo negro, letras blancas, auto-scroll
  con velocidad ajustable, tamaño de letra y modo espejado).
- Columna "Guion" sumada al import/export de Excel y a
  IMPORT_DIFF_FIELDS (participa en preview/diff/undo).
- Plantilla descargable actualizada con la columna nueva + instrucciones.
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
+++ b/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A50"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -626,7 +626,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
@@ -696,103 +695,117 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-    </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>GUION Y TELEPROMPTER (opcional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>• Columna 'Guion': el texto completo para leer mientras se graba la pieza. Adentro del hub, cada contenido tiene un botón '📺 Abrir teleprompter' que lo muestra a pantalla completa (fondo negro, letras blancas, auto-scroll).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>VALORES VÁLIDOS POR COLUMNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
+          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
+          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
+          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
+          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
+          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
-        </is>
-      </c>
+      <c r="A49" s="2" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos, asignación a alguien del equipo) se completan después, ya adentro del hub.</t>
+          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos) se completan después, ya adentro del hub.</t>
         </is>
       </c>
     </row>
@@ -807,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -825,7 +838,7 @@
     <col width="40" customWidth="1" min="13" max="13"/>
     <col width="40" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="16" max="16"/>
     <col width="32" customWidth="1" min="17" max="17"/>
     <col width="30" customWidth="1" min="18" max="18"/>
     <col width="22" customWidth="1" min="20" max="20"/>
@@ -909,30 +922,35 @@
       </c>
       <c r="P1" s="4" t="inlineStr">
         <is>
+          <t>Guion</t>
+        </is>
+      </c>
+      <c r="Q1" s="4" t="inlineStr">
+        <is>
           <t>Pauta</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>Link pieza terminada</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>Link material de referencia</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>Notas internas</t>
         </is>
       </c>
-      <c r="T1" s="7" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>Asignado a</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>Pilar / fase (referencia interna, NO se sube al hub)</t>
         </is>
@@ -1014,19 +1032,19 @@
           <t>Ej: Plano 1: producto entero sobre mesa de madera clara. Plano 2: primer plano de la mano abriendo el envase. Plano 3: producto servido, luz cálida.</t>
         </is>
       </c>
-      <c r="P2" s="5" t="inlineStr">
+      <c r="Q2" s="5" t="inlineStr">
         <is>
           <t>Solo orgánico</t>
         </is>
       </c>
-      <c r="Q2" s="5" t="inlineStr"/>
       <c r="R2" s="5" t="inlineStr"/>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="S2" s="5" t="inlineStr"/>
+      <c r="T2" s="5" t="inlineStr">
         <is>
           <t>Ejemplo de fila — borrala y cargá tus propios contenidos.</t>
         </is>
       </c>
-      <c r="U2" s="5" t="inlineStr">
+      <c r="V2" s="5" t="inlineStr">
         <is>
           <t>Septiembre · Ejemplo</t>
         </is>

</xml_diff>

<commit_message>
Importar Excel: leer la hoja de datos (no 'Instrucciones') y plantillas con los datos en la primera hoja
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QtS8C8GC6PUTqNPYTJiSZE
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
+++ b/plantillas/Plantilla_Contenidos_Hub_COSMART.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Contenidos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contenidos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,348 +478,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PLANTILLA BASE — Carga de contenidos al COSMART Marketing Hub</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Esta hoja ('Contenidos') tiene una columna por cada campo del formulario 'Nuevo contenido' del hub.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Completá una fila por cada pieza de contenido (una fila = un posteo en una plataforma).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>CÓMO FUNCIONA LA IMPORTACIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>1. En el hub, sección Contenidos → botón 'Importar Excel'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2. Subís este archivo (sin cambiar los nombres de las columnas del encabezado, fila 1).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>3. El hub identifica cada fila por Título + Cuenta:</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Si NO existe todavía → se agrega como contenido nuevo, estado 'Idea' salvo que indiques otro.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Si YA existe y no cambió nada → se deja como está, no se duplica.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Si YA existe y algún campo cambió → se muestra qué cambió (antes/después) y elegís, fila por fila,</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     'Reemplazar' (actualiza ese contenido con los datos nuevos) u 'Omitir' (lo deja como está).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>4. Podés reordenar las columnas — el sistema las identifica por el NOMBRE del encabezado, no por posición.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>5. No borres ni renombres la fila 1 (encabezados). Podés agregar columnas propias al final, se ignoran al subir.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>CAMPOS OBLIGATORIOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>• Título del contenido</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>• Estado (si lo dejás vacío, se sube como 'Idea')</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>• Cuenta (el handle configurado en el hub, ej: minamiworldok)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>• Plataformas (al menos una)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>• Formato (al menos uno)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>ASIGNAR EL CONTENIDO A ALGUIEN (opcional)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>• Columna 'Asignado a': escribí el nombre o el email de a quién se lo querés asignar -- tiene que ser el contacto del cliente o alguien del equipo ya agregado a este cliente en el hub. Si no coincide con nadie, se sube sin asignar (no da error).</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>CAMPOS QUE ACEPTAN VARIOS VALORES (separar con coma dentro de la misma celda)</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Plataformas, Ubicación, Formato, Dimensiones — ej: 'Instagram, TikTok' o 'Feed, Story'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>COPY vs. TEXTO EN PANTALLA — son dos cosas distintas, no las mezcles</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>• Copy: el texto de la descripción/caption del posteo (lo que se lee debajo, en el feed).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>• Texto en pantalla: el texto que aparece escrito DENTRO de la pieza (imagen o video).</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>• Prompt sugerido para IA: si esa pieza se va a generar con inteligencia artificial, el prompt sugerido para armarla (opcional).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>• Sugerencia de pieza creativa: cómo se imagina la pieza visualmente -- descripción de la imagen, o secuencia de escenas/planos si es un video (distinto del prompt de IA de arriba, es para guiar a quien diseña/filma, se use o no IA).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>GUION Y TELEPROMPTER (opcional)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>• Columna 'Guion': el texto completo para leer mientras se graba la pieza. Adentro del hub, cada contenido tiene un botón '📺 Abrir teleprompter' que lo muestra a pantalla completa (fondo negro, letras blancas, auto-scroll).</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>VALORES VÁLIDOS POR COLUMNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos) se completan después, ya adentro del hub.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:V2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1053,4 +711,346 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A53"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PLANTILLA BASE — Carga de contenidos al COSMART Marketing Hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Esta hoja ('Contenidos') tiene una columna por cada campo del formulario 'Nuevo contenido' del hub.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Completá una fila por cada pieza de contenido (una fila = un posteo en una plataforma).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CÓMO FUNCIONA LA IMPORTACIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1. En el hub, sección Contenidos → botón 'Importar Excel'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2. Subís este archivo (sin cambiar los nombres de las columnas del encabezado, fila 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>3. El hub identifica cada fila por Título + Cuenta:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Si NO existe todavía → se agrega como contenido nuevo, estado 'Idea' salvo que indiques otro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Si YA existe y no cambió nada → se deja como está, no se duplica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Si YA existe y algún campo cambió → se muestra qué cambió (antes/después) y elegís, fila por fila,</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     'Reemplazar' (actualiza ese contenido con los datos nuevos) u 'Omitir' (lo deja como está).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>4. Podés reordenar las columnas — el sistema las identifica por el NOMBRE del encabezado, no por posición.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>5. No borres ni renombres la fila 1 (encabezados). Podés agregar columnas propias al final, se ignoran al subir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CAMPOS OBLIGATORIOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>• Título del contenido</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>• Estado (si lo dejás vacío, se sube como 'Idea')</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>• Cuenta (el handle configurado en el hub, ej: minamiworldok)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>• Plataformas (al menos una)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>• Formato (al menos uno)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>ASIGNAR EL CONTENIDO A ALGUIEN (opcional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>• Columna 'Asignado a': escribí el nombre o el email de a quién se lo querés asignar -- tiene que ser el contacto del cliente o alguien del equipo ya agregado a este cliente en el hub. Si no coincide con nadie, se sube sin asignar (no da error).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>CAMPOS QUE ACEPTAN VARIOS VALORES (separar con coma dentro de la misma celda)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Plataformas, Ubicación, Formato, Dimensiones — ej: 'Instagram, TikTok' o 'Feed, Story'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>COPY vs. TEXTO EN PANTALLA — son dos cosas distintas, no las mezcles</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>• Copy: el texto de la descripción/caption del posteo (lo que se lee debajo, en el feed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>• Texto en pantalla: el texto que aparece escrito DENTRO de la pieza (imagen o video).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>• Prompt sugerido para IA: si esa pieza se va a generar con inteligencia artificial, el prompt sugerido para armarla (opcional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>• Sugerencia de pieza creativa: cómo se imagina la pieza visualmente -- descripción de la imagen, o secuencia de escenas/planos si es un video (distinto del prompt de IA de arriba, es para guiar a quien diseña/filma, se use o no IA).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>GUION Y TELEPROMPTER (opcional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>• Columna 'Guion': el texto completo para leer mientras se graba la pieza. Adentro del hub, cada contenido tiene un botón '📺 Abrir teleprompter' que lo muestra a pantalla completa (fondo negro, letras blancas, auto-scroll).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>VALORES VÁLIDOS POR COLUMNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Estado: Idea, En proceso, En revisión, Aprobado, Programado, Publicado</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Plataformas: Instagram, Facebook, LinkedIn, Twitter / X, TikTok, YouTube, Sitio Web, Blog</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Ubicación según plataforma — Instagram/Facebook: Feed, Story, Reel, Carrusel · TikTok: Feed, Story · YouTube: Feed, Shorts · LinkedIn/Twitter: Feed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Formato según plataforma — Instagram: Imagen, Video, Reel, Carrusel, Story, GIF · TikTok: Video · YouTube: Video · LinkedIn: Imagen, Video, Carrusel, Documento</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Dimensiones: 1:1, 4:5, 9:16, 16:9, 1.91:1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Eje de comunicación: Institucional, Entretenimiento, Comercial, Interacción, Educativo, Inspiracional</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Tipo de contenido: Informativo, Promocional, Sorteo, Viral, Evento, Celebración, Tutorial</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: Notoriedad, Engagement, Alcance, Conversión, Tráfico</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Pauta: Solo orgánico, Sí – Dark post, Sí – Dark + orgánico</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Fecha de publicación: formato AAAA-MM-DD (ej: 2026-08-15). Si Excel la formatea como fecha, funciona igual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>La última columna ('Pilar / fase') es solo para planificación estratégica interna: no es un campo del hub y se descarta al importar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Los campos que no están en esta plantilla (comentarios, archivos adjuntos) se completan después, ya adentro del hub.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>